<commit_message>
Control board BOM for 500 and 1000 boards added.
</commit_message>
<xml_diff>
--- a/Deliverables/Control_Board/BOM/Altium Generated BOM Control_Board.xlsx
+++ b/Deliverables/Control_Board/BOM/Altium Generated BOM Control_Board.xlsx
@@ -1,33 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\ChrisitanRaun-AnnanasMotor\Design-Files\ControlBoard-DesignFiles\Project Outputs for Control_Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ChrisitanRaun-AnnanasMotor\Deliverables\Control_Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{41F73E86-7770-4D62-BA0C-1900C44A77A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="14430"/>
+    <workbookView xWindow="7035" yWindow="300" windowWidth="10335" windowHeight="10620" xr2:uid="{CF46F1DC-E390-44DE-9ADC-5B141A9D882E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Control_Board" sheetId="1" r:id="rId1"/>
+    <sheet name="Altium Generated BOM Control_Bo" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Control_Board!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Altium Generated BOM Control_Bo'!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="124">
   <si>
     <t>Comment</t>
   </si>
@@ -155,13 +163,16 @@
     <t>PH254P1x12SMRA-100_1</t>
   </si>
   <si>
-    <t>PHF254SMD-x</t>
-  </si>
-  <si>
-    <t>P=2.54mm Female Headers,SMD,ROHS</t>
+    <t>95278-101A26LF</t>
+  </si>
+  <si>
+    <t>CONN HEADER SMD 26POS 2.54MM</t>
   </si>
   <si>
     <t>J3</t>
+  </si>
+  <si>
+    <t>Amphenol ICC (FCI)</t>
   </si>
   <si>
     <t>MLB1608-201P1A(f)</t>
@@ -401,7 +412,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -498,7 +509,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -510,7 +521,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -557,6 +568,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -592,6 +620,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -743,7 +788,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D6868A-9F0A-4516-8463-638A210F92F4}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -958,93 +1003,93 @@
         <v>1</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>45</v>
-      </c>
       <c r="E10" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F10" s="4">
         <v>5</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>49</v>
-      </c>
       <c r="F11" s="4">
         <v>1</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>54</v>
       </c>
       <c r="F12" s="4">
         <v>3</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F13" s="4">
         <v>3</v>
@@ -1053,19 +1098,19 @@
     </row>
     <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F14" s="4">
         <v>12</v>
@@ -1076,19 +1121,19 @@
     </row>
     <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F15" s="4">
         <v>3</v>
@@ -1099,19 +1144,19 @@
     </row>
     <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F16" s="4">
         <v>1</v>
@@ -1122,19 +1167,19 @@
     </row>
     <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F17" s="4">
         <v>4</v>
@@ -1145,19 +1190,19 @@
     </row>
     <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F18" s="4">
         <v>1</v>
@@ -1168,19 +1213,19 @@
     </row>
     <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F19" s="4">
         <v>2</v>
@@ -1191,19 +1236,19 @@
     </row>
     <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F20" s="4">
         <v>1</v>
@@ -1214,19 +1259,19 @@
     </row>
     <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>92</v>
-      </c>
       <c r="E21" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F21" s="4">
         <v>5</v>
@@ -1235,163 +1280,163 @@
     </row>
     <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="E22" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F22" s="4">
         <v>1</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B23" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>99</v>
-      </c>
       <c r="E23" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F23" s="4">
         <v>1</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>103</v>
-      </c>
       <c r="E24" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F24" s="4">
         <v>1</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>107</v>
-      </c>
       <c r="E25" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F25" s="4">
         <v>1</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>111</v>
-      </c>
       <c r="E26" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F26" s="4">
         <v>1</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>115</v>
-      </c>
       <c r="E27" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F27" s="4">
         <v>1</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>119</v>
-      </c>
       <c r="E28" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F28" s="4">
         <v>1</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>